<commit_message>
Integra las referencias vigentes y sus casos de validación
</commit_message>
<xml_diff>
--- a/DIPs References.xlsx
+++ b/DIPs References.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://copaairlines.sharepoint.com/teams/VP_Tecnica/dacre/records/DPPT Library/12 - DIP Audit Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{157EDD76-58A3-4522-9FC2-76B2E858213E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="990" documentId="8_{6C06C099-B655-452B-86A2-4DC3BD5D41B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BFA48B0-AA45-4193-8D7A-6236C73D1E8A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="270">
   <si>
     <t>TYPE</t>
   </si>
@@ -349,12 +349,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">1 FC IF PRESSURE IS BETWEEN 50-100 PSI ABOVE THE MINIMUM DISPATCH PRESSURE. 1 DAY IF PRESSURE IS BETWEEN 100-200 PSI, ABOVE THE MINIMUM DISPATCH PRESSURE. </t>
     </r>
     <r>
@@ -666,6 +660,12 @@
     <t>TASKCARD B737-73-1-0001-U-JIC</t>
   </si>
   <si>
+    <t>FUEL PUMP</t>
+  </si>
+  <si>
+    <t>FUEL PUMP PAD PLUG</t>
+  </si>
+  <si>
     <t>STRUCTURES</t>
   </si>
   <si>
@@ -762,40 +762,10 @@
     <t>LIGHTNING STRIKE FOUND</t>
   </si>
   <si>
-    <t>SRM 53-00-01</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">10 FC, 350 FC OR BEFORE NEXT REVENUE FLIGHT. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CONSULT SRM 53-00-01</t>
-    </r>
-  </si>
-  <si>
-    <t>LIGHTNING</t>
-  </si>
-  <si>
-    <t>LIGHTNING STRIKE PHASE II</t>
-  </si>
-  <si>
-    <t>AMM TASK 05-51-19-210-804</t>
-  </si>
-  <si>
-    <t>50 FC</t>
+    <t>SRM 53-00-01-1A-1</t>
+  </si>
+  <si>
+    <t>350 FC</t>
   </si>
   <si>
     <t>CHEMICAL OXYGEN GENERATOR (PSU / ASU / LAV) LIFE LIMIT - CLOSE TO DUE DATE</t>
@@ -904,7 +874,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -946,13 +916,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -1011,7 +975,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1025,27 +989,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1054,21 +1021,39 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -1078,15 +1063,27 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
@@ -1117,8 +1114,8 @@
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>438150</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>111125</xdr:rowOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>187325</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1473,7 +1470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="13.5703125" style="3" customWidth="1"/>
@@ -1518,7 +1515,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="29.1">
+    <row r="2" spans="1:11" ht="30.75">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -1547,7 +1544,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="29.1">
+    <row r="3" spans="1:11" ht="30.75">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1573,11 +1570,11 @@
         <v>18</v>
       </c>
       <c r="I3" s="1"/>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="101.45">
+    <row r="4" spans="1:11" ht="106.5">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -1603,11 +1600,11 @@
         <v>23</v>
       </c>
       <c r="I4" s="1"/>
-      <c r="K4" s="11" t="s">
+      <c r="K4" s="8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="29.1">
+    <row r="5" spans="1:11" ht="30.75">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1634,7 +1631,7 @@
       </c>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:11" ht="29.1">
+    <row r="6" spans="1:11" ht="30.75">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -1661,7 +1658,7 @@
       </c>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" spans="1:11" ht="29.1">
+    <row r="7" spans="1:11" ht="30.75">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -1688,7 +1685,7 @@
       </c>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:11" ht="29.1">
+    <row r="8" spans="1:11" ht="30.75">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -1715,7 +1712,7 @@
       </c>
       <c r="I8" s="1"/>
     </row>
-    <row r="9" spans="1:11" ht="29.1">
+    <row r="9" spans="1:11" ht="30.75">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1742,7 +1739,7 @@
       </c>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:11" ht="29.1">
+    <row r="10" spans="1:11" ht="30.75">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1769,7 +1766,7 @@
       </c>
       <c r="I10" s="1"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" ht="15">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1796,7 +1793,7 @@
       </c>
       <c r="I11" s="1"/>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" ht="15">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -1823,7 +1820,7 @@
       </c>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" ht="15">
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1850,7 +1847,7 @@
       </c>
       <c r="I13" s="1"/>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" ht="15">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -1877,7 +1874,7 @@
       </c>
       <c r="I14" s="1"/>
     </row>
-    <row r="15" spans="1:11" ht="29.1">
+    <row r="15" spans="1:11" ht="30.75">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
@@ -1904,7 +1901,7 @@
       </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" ht="30.75">
       <c r="A16" s="1" t="s">
         <v>9</v>
       </c>
@@ -1931,7 +1928,7 @@
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" ht="15">
       <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
@@ -1958,7 +1955,7 @@
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" ht="15">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
@@ -1985,7 +1982,7 @@
       </c>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" ht="15">
       <c r="A19" s="1" t="s">
         <v>9</v>
       </c>
@@ -2012,7 +2009,7 @@
       </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" ht="15">
       <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
@@ -2039,7 +2036,7 @@
       </c>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" ht="15">
       <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
@@ -2066,7 +2063,7 @@
       </c>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" ht="15">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
@@ -2093,7 +2090,7 @@
       </c>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" ht="15">
       <c r="A23" s="1" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +2117,7 @@
       </c>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" ht="15">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -2147,7 +2144,7 @@
       </c>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" ht="15">
       <c r="A25" s="1" t="s">
         <v>9</v>
       </c>
@@ -2174,7 +2171,7 @@
       </c>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" ht="15">
       <c r="A26" s="1" t="s">
         <v>9</v>
       </c>
@@ -2201,7 +2198,7 @@
       </c>
       <c r="I26" s="1"/>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" ht="15">
       <c r="A27" s="1" t="s">
         <v>9</v>
       </c>
@@ -2228,7 +2225,7 @@
       </c>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" ht="15">
       <c r="A28" s="1" t="s">
         <v>9</v>
       </c>
@@ -2257,7 +2254,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="101.45">
+    <row r="29" spans="1:9" ht="106.5">
       <c r="A29" s="1" t="s">
         <v>9</v>
       </c>
@@ -2279,12 +2276,12 @@
       <c r="G29" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H29" s="10" t="s">
         <v>89</v>
       </c>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:9" ht="101.45">
+    <row r="30" spans="1:9" ht="106.5">
       <c r="A30" s="1" t="s">
         <v>9</v>
       </c>
@@ -2306,12 +2303,12 @@
       <c r="G30" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="10" t="s">
         <v>89</v>
       </c>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="1:9" ht="72.599999999999994">
+    <row r="31" spans="1:9" ht="76.5">
       <c r="A31" s="1" t="s">
         <v>9</v>
       </c>
@@ -2338,7 +2335,7 @@
       </c>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" ht="15">
       <c r="A32" s="1" t="s">
         <v>9</v>
       </c>
@@ -2387,12 +2384,12 @@
       <c r="G33" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="H33" s="8" t="s">
+      <c r="H33" s="6" t="s">
         <v>102</v>
       </c>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" ht="15">
       <c r="A34" s="1" t="s">
         <v>9</v>
       </c>
@@ -2419,7 +2416,7 @@
       </c>
       <c r="I34" s="1"/>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" ht="15">
       <c r="A35" s="1" t="s">
         <v>9</v>
       </c>
@@ -2446,7 +2443,7 @@
       </c>
       <c r="I35" s="1"/>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" ht="15">
       <c r="A36" s="1" t="s">
         <v>9</v>
       </c>
@@ -2473,7 +2470,7 @@
       </c>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" ht="15">
       <c r="A37" s="1" t="s">
         <v>9</v>
       </c>
@@ -2500,7 +2497,7 @@
       </c>
       <c r="I37" s="1"/>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" ht="15">
       <c r="A38" s="1" t="s">
         <v>9</v>
       </c>
@@ -2527,7 +2524,7 @@
       </c>
       <c r="I38" s="1"/>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" ht="15">
       <c r="A39" s="1" t="s">
         <v>9</v>
       </c>
@@ -2554,7 +2551,7 @@
       </c>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" ht="15">
       <c r="A40" s="1" t="s">
         <v>9</v>
       </c>
@@ -2581,7 +2578,7 @@
       </c>
       <c r="I40" s="1"/>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" ht="15">
       <c r="A41" s="1" t="s">
         <v>9</v>
       </c>
@@ -2608,7 +2605,7 @@
       </c>
       <c r="I41" s="1"/>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" ht="15">
       <c r="A42" s="1" t="s">
         <v>9</v>
       </c>
@@ -2635,7 +2632,7 @@
       </c>
       <c r="I42" s="1"/>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" ht="15">
       <c r="A43" s="1" t="s">
         <v>9</v>
       </c>
@@ -2662,7 +2659,7 @@
       </c>
       <c r="I43" s="1"/>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" ht="15">
       <c r="A44" s="1" t="s">
         <v>9</v>
       </c>
@@ -2689,7 +2686,7 @@
       </c>
       <c r="I44" s="1"/>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" ht="15">
       <c r="A45" s="1" t="s">
         <v>9</v>
       </c>
@@ -2716,7 +2713,7 @@
       </c>
       <c r="I45" s="1"/>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" ht="15">
       <c r="A46" s="1" t="s">
         <v>9</v>
       </c>
@@ -2743,7 +2740,7 @@
       </c>
       <c r="I46" s="1"/>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" ht="15">
       <c r="A47" s="1" t="s">
         <v>9</v>
       </c>
@@ -2768,7 +2765,7 @@
       </c>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" ht="15">
       <c r="A48" s="1" t="s">
         <v>9</v>
       </c>
@@ -2791,7 +2788,7 @@
       </c>
       <c r="I48" s="1"/>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" ht="15">
       <c r="A49" s="1" t="s">
         <v>9</v>
       </c>
@@ -2814,7 +2811,7 @@
       </c>
       <c r="I49" s="1"/>
     </row>
-    <row r="50" spans="1:9">
+    <row r="50" spans="1:9" ht="15">
       <c r="A50" s="1" t="s">
         <v>9</v>
       </c>
@@ -2837,7 +2834,7 @@
       </c>
       <c r="I50" s="1"/>
     </row>
-    <row r="51" spans="1:9">
+    <row r="51" spans="1:9" ht="15">
       <c r="A51" s="1" t="s">
         <v>9</v>
       </c>
@@ -2860,7 +2857,7 @@
       </c>
       <c r="I51" s="1"/>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:9" ht="15">
       <c r="A52" s="1" t="s">
         <v>9</v>
       </c>
@@ -2883,7 +2880,7 @@
       </c>
       <c r="I52" s="1"/>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:9" ht="15">
       <c r="A53" s="1" t="s">
         <v>9</v>
       </c>
@@ -2906,7 +2903,7 @@
       </c>
       <c r="I53" s="1"/>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:9" ht="15">
       <c r="A54" s="1" t="s">
         <v>137</v>
       </c>
@@ -2935,7 +2932,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="29.1">
+    <row r="55" spans="1:9" ht="30.75">
       <c r="A55" s="1" t="s">
         <v>137</v>
       </c>
@@ -2962,7 +2959,7 @@
       </c>
       <c r="I55" s="1"/>
     </row>
-    <row r="56" spans="1:9">
+    <row r="56" spans="1:9" ht="15">
       <c r="A56" s="1" t="s">
         <v>137</v>
       </c>
@@ -2989,7 +2986,7 @@
       </c>
       <c r="I56" s="1"/>
     </row>
-    <row r="57" spans="1:9">
+    <row r="57" spans="1:9" ht="15">
       <c r="A57" s="1" t="s">
         <v>137</v>
       </c>
@@ -3018,7 +3015,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="58" spans="1:9">
+    <row r="58" spans="1:9" ht="15">
       <c r="A58" s="1" t="s">
         <v>137</v>
       </c>
@@ -3045,7 +3042,7 @@
       </c>
       <c r="I58" s="1"/>
     </row>
-    <row r="59" spans="1:9" ht="29.1">
+    <row r="59" spans="1:9" ht="30.75">
       <c r="A59" s="1" t="s">
         <v>137</v>
       </c>
@@ -3072,7 +3069,7 @@
       </c>
       <c r="I59" s="1"/>
     </row>
-    <row r="60" spans="1:9" ht="43.5">
+    <row r="60" spans="1:9" ht="45.75">
       <c r="A60" s="1" t="s">
         <v>137</v>
       </c>
@@ -3099,7 +3096,7 @@
       </c>
       <c r="I60" s="1"/>
     </row>
-    <row r="61" spans="1:9" ht="43.5">
+    <row r="61" spans="1:9" ht="45.75">
       <c r="A61" s="1" t="s">
         <v>137</v>
       </c>
@@ -3121,12 +3118,12 @@
       <c r="G61" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="H61" s="6" t="s">
+      <c r="H61" s="5" t="s">
         <v>167</v>
       </c>
       <c r="I61" s="1"/>
     </row>
-    <row r="62" spans="1:9" ht="29.1">
+    <row r="62" spans="1:9" ht="30.75">
       <c r="A62" s="1" t="s">
         <v>137</v>
       </c>
@@ -3153,7 +3150,7 @@
       </c>
       <c r="I62" s="1"/>
     </row>
-    <row r="63" spans="1:9" ht="29.1">
+    <row r="63" spans="1:9" ht="30.75">
       <c r="A63" s="1" t="s">
         <v>137</v>
       </c>
@@ -3180,7 +3177,7 @@
       </c>
       <c r="I63" s="1"/>
     </row>
-    <row r="64" spans="1:9" ht="29.1">
+    <row r="64" spans="1:9" ht="30.75">
       <c r="A64" s="1" t="s">
         <v>137</v>
       </c>
@@ -3209,7 +3206,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="29.1">
+    <row r="65" spans="1:9" ht="30.75">
       <c r="A65" s="1" t="s">
         <v>137</v>
       </c>
@@ -3238,7 +3235,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="29.1">
+    <row r="66" spans="1:9" ht="30.75">
       <c r="A66" s="1" t="s">
         <v>137</v>
       </c>
@@ -3267,7 +3264,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="67" spans="1:9">
+    <row r="67" spans="1:9" ht="15">
       <c r="A67" s="1" t="s">
         <v>137</v>
       </c>
@@ -3294,7 +3291,7 @@
       </c>
       <c r="I67" s="1"/>
     </row>
-    <row r="68" spans="1:9" ht="43.5">
+    <row r="68" spans="1:9" ht="45.75">
       <c r="A68" s="1" t="s">
         <v>137</v>
       </c>
@@ -3323,34 +3320,34 @@
         <v>189</v>
       </c>
     </row>
-    <row r="69" spans="1:9">
-      <c r="A69" s="5" t="s">
+    <row r="69" spans="1:9" ht="15">
+      <c r="A69" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="C69" s="5">
+      <c r="C69" s="11">
         <v>71</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E69" s="5" t="s">
+      <c r="E69" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="F69" s="5" t="s">
+      <c r="F69" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="G69" s="5" t="s">
+      <c r="G69" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="H69" s="5" t="s">
+      <c r="H69" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="I69" s="5"/>
-    </row>
-    <row r="70" spans="1:9">
+      <c r="I69" s="11"/>
+    </row>
+    <row r="70" spans="1:9" ht="15">
       <c r="A70" s="1" t="s">
         <v>137</v>
       </c>
@@ -3379,7 +3376,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="71" spans="1:9">
+    <row r="71" spans="1:9" ht="15">
       <c r="A71" s="1" t="s">
         <v>137</v>
       </c>
@@ -3406,7 +3403,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="72" spans="1:9">
+    <row r="72" spans="1:9" ht="15">
       <c r="A72" s="1" t="s">
         <v>137</v>
       </c>
@@ -3435,124 +3432,120 @@
         <v>153</v>
       </c>
     </row>
-    <row r="73" spans="1:9">
-      <c r="A73" s="1" t="s">
+    <row r="73" spans="1:9" ht="15">
+      <c r="A73" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="B73" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="C73" s="13">
+        <v>71</v>
+      </c>
+      <c r="D73" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E73" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="C73" s="1">
+      <c r="F73" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="G73" s="13"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="13"/>
+    </row>
+    <row r="74" spans="1:9" ht="15">
+      <c r="A74" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C74" s="1">
         <v>56</v>
       </c>
-      <c r="D73" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G73" s="1" t="s">
+      <c r="D74" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="76.5">
+      <c r="A75" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="H73" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="I73" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" ht="57.95">
-      <c r="A74" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B74" s="1" t="s">
+      <c r="B75" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C75" s="1">
+        <v>54</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="30.75">
+      <c r="A76" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C76" s="1">
+        <v>56</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="H76" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="C74" s="1">
-        <v>54</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E74" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="G74" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="H74" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I74" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" ht="29.1">
-      <c r="A75" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C75" s="1">
-        <v>56</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="H75" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="I75" s="1"/>
-    </row>
-    <row r="76" spans="1:9">
-      <c r="A76" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C76" s="1">
-        <v>52</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E76" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G76" s="1" t="s">
+      <c r="I76" s="1"/>
+    </row>
+    <row r="77" spans="1:9" ht="15">
+      <c r="A77" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B77" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="H76" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I76" s="1"/>
-    </row>
-    <row r="77" spans="1:9" ht="30.75">
-      <c r="A77" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>212</v>
       </c>
       <c r="C77" s="1">
         <v>52</v>
@@ -3560,7 +3553,7 @@
       <c r="D77" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E77" s="4" t="s">
+      <c r="E77" s="1" t="s">
         <v>215</v>
       </c>
       <c r="F77" s="1" t="s">
@@ -3570,43 +3563,43 @@
         <v>216</v>
       </c>
       <c r="H77" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I77" s="1"/>
+    </row>
+    <row r="78" spans="1:9" ht="30.75">
+      <c r="A78" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C78" s="1">
+        <v>52</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E78" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="I77" s="1"/>
-    </row>
-    <row r="78" spans="1:9">
-      <c r="A78" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B78" s="1" t="s">
+      <c r="F78" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G78" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="C78" s="1">
-        <v>51</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E78" s="1" t="s">
+      <c r="H78" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="F78" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G78" s="1" t="s">
+      <c r="I78" s="1"/>
+    </row>
+    <row r="79" spans="1:9" ht="15">
+      <c r="A79" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B79" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="H78" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="I78" s="1"/>
-    </row>
-    <row r="79" spans="1:9" ht="29.1">
-      <c r="A79" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>201</v>
       </c>
       <c r="C79" s="1">
         <v>51</v>
@@ -3615,28 +3608,28 @@
         <v>11</v>
       </c>
       <c r="E79" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G79" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="F79" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G79" s="1" t="s">
+      <c r="H79" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="H79" s="1" t="s">
+      <c r="I79" s="1"/>
+    </row>
+    <row r="80" spans="1:9" ht="30.75">
+      <c r="A80" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="I79" s="1"/>
-    </row>
-    <row r="80" spans="1:9">
-      <c r="A80" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>212</v>
-      </c>
       <c r="C80" s="1">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>11</v>
@@ -3651,389 +3644,389 @@
         <v>225</v>
       </c>
       <c r="H80" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="I80" s="1"/>
+    </row>
+    <row r="81" spans="1:9" ht="15">
+      <c r="A81" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C81" s="1">
+        <v>52</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E81" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="I80" s="1"/>
-    </row>
-    <row r="81" spans="1:9" ht="30.75">
-      <c r="A81" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="C81" s="1">
+      <c r="F81" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="I81" s="1"/>
+    </row>
+    <row r="82" spans="1:9" ht="30.75">
+      <c r="A82" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C82" s="1">
         <v>57</v>
       </c>
-      <c r="D81" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="H81" s="1" t="s">
+      <c r="D82" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E82" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="I81" s="1"/>
-    </row>
-    <row r="82" spans="1:9" ht="45.75">
-      <c r="A82" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B82" s="1" t="s">
+      <c r="F82" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G82" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C82" s="1">
-        <v>53</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E82" s="1" t="s">
+      <c r="H82" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="H82" s="8" t="s">
-        <v>233</v>
       </c>
       <c r="I82" s="1"/>
     </row>
     <row r="83" spans="1:9" ht="15">
       <c r="A83" s="1" t="s">
-        <v>9</v>
+        <v>202</v>
       </c>
       <c r="B83" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C83" s="1">
+        <v>53</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G83" t="s">
         <v>234</v>
       </c>
-      <c r="C83" s="1">
+      <c r="H83" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="I83" s="1"/>
+    </row>
+    <row r="84" spans="1:9" ht="60.75">
+      <c r="A84" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C84" s="2">
+        <v>35</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I84" s="12"/>
+    </row>
+    <row r="85" spans="1:9" ht="106.5">
+      <c r="A85" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I85" s="12"/>
+    </row>
+    <row r="86" spans="1:9" ht="45.75">
+      <c r="A86" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C86" s="2">
+        <v>27</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I86" s="12"/>
+    </row>
+    <row r="87" spans="1:9" ht="60.75">
+      <c r="A87" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C87" s="2">
+        <v>46</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="H87" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="I87" s="12"/>
+    </row>
+    <row r="88" spans="1:9" ht="106.5">
+      <c r="A88" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C88" s="2">
+        <v>77</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I88" s="12"/>
+    </row>
+    <row r="89" spans="1:9" ht="106.5">
+      <c r="A89" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C89" s="2">
+        <v>79</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H89" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="I89" s="12"/>
+    </row>
+    <row r="90" spans="1:9" ht="60.75">
+      <c r="A90" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C90" s="2">
+        <v>28</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="I90" s="12"/>
+    </row>
+    <row r="91" spans="1:9" ht="91.5">
+      <c r="A91" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C91" s="2">
+        <v>28</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I91" s="12"/>
+    </row>
+    <row r="92" spans="1:9" ht="30.75">
+      <c r="A92" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C92" s="2">
+        <v>54</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="I92" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="45.75">
+      <c r="A93" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C93" s="2">
+        <v>32</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H93" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="I93" s="12"/>
+    </row>
+    <row r="94" spans="1:9" ht="30.75">
+      <c r="A94" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C94" s="2">
         <v>5</v>
       </c>
-      <c r="D83" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="F83" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G83" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="H83" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="I83" s="1"/>
-    </row>
-    <row r="84" spans="1:9" ht="51.95">
-      <c r="A84" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B84" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="C84" s="12">
-        <v>35</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E84" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="F84" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G84" s="12" t="s">
-        <v>239</v>
-      </c>
-      <c r="H84" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I84" s="13"/>
-    </row>
-    <row r="85" spans="1:9" ht="78">
-      <c r="A85" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="B85" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="C85" s="12" t="s">
-        <v>241</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E85" s="12" t="s">
-        <v>242</v>
-      </c>
-      <c r="F85" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G85" s="12" t="s">
-        <v>243</v>
-      </c>
-      <c r="H85" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="I85" s="13"/>
-    </row>
-    <row r="86" spans="1:9" ht="26.1">
-      <c r="A86" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B86" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="C86" s="12">
-        <v>27</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E86" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="F86" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G86" s="12" t="s">
-        <v>245</v>
-      </c>
-      <c r="H86" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="I86" s="13"/>
-    </row>
-    <row r="87" spans="1:9" ht="39">
-      <c r="A87" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B87" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="C87" s="12">
-        <v>46</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E87" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="F87" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G87" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="H87" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="I87" s="13"/>
-    </row>
-    <row r="88" spans="1:9" ht="78">
-      <c r="A88" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="B88" s="12" t="s">
-        <v>249</v>
-      </c>
-      <c r="C88" s="12">
-        <v>77</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E88" s="12" t="s">
-        <v>250</v>
-      </c>
-      <c r="F88" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="G88" s="12" t="s">
-        <v>251</v>
-      </c>
-      <c r="H88" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="I88" s="13"/>
-    </row>
-    <row r="89" spans="1:9" ht="78">
-      <c r="A89" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="B89" s="12" t="s">
-        <v>249</v>
-      </c>
-      <c r="C89" s="12">
-        <v>79</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E89" s="12" t="s">
-        <v>252</v>
-      </c>
-      <c r="F89" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="G89" s="12" t="s">
-        <v>253</v>
-      </c>
-      <c r="H89" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="I89" s="13"/>
-    </row>
-    <row r="90" spans="1:9" ht="51.95">
-      <c r="A90" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B90" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C90" s="12">
-        <v>28</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E90" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="F90" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G90" s="12" t="s">
-        <v>256</v>
-      </c>
-      <c r="H90" s="12" t="s">
-        <v>257</v>
-      </c>
-      <c r="I90" s="13"/>
-    </row>
-    <row r="91" spans="1:9" ht="65.099999999999994">
-      <c r="A91" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B91" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C91" s="12">
-        <v>28</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E91" s="12" t="s">
-        <v>258</v>
-      </c>
-      <c r="F91" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G91" s="12" t="s">
-        <v>259</v>
-      </c>
-      <c r="H91" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="I91" s="13"/>
-    </row>
-    <row r="92" spans="1:9" ht="26.1">
-      <c r="A92" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="B92" s="12" t="s">
-        <v>261</v>
-      </c>
-      <c r="C92" s="12">
-        <v>54</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E92" s="12" t="s">
-        <v>262</v>
-      </c>
-      <c r="F92" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G92" s="12" t="s">
-        <v>263</v>
-      </c>
-      <c r="H92" s="12" t="s">
-        <v>264</v>
-      </c>
-      <c r="I92" s="12" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9" ht="39">
-      <c r="A93" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B93" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="C93" s="12">
-        <v>32</v>
-      </c>
-      <c r="D93" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E93" s="12" t="s">
-        <v>265</v>
-      </c>
-      <c r="F93" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G93" s="12" t="s">
-        <v>266</v>
-      </c>
-      <c r="H93" s="12" t="s">
+      <c r="D94" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="I93" s="13"/>
-    </row>
-    <row r="94" spans="1:9" ht="26.1">
-      <c r="A94" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B94" s="12" t="s">
+      <c r="F94" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G94" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C94" s="12">
-        <v>5</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E94" s="12" t="s">
+      <c r="H94" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="F94" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G94" s="12" t="s">
-        <v>270</v>
-      </c>
-      <c r="H94" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="I94" s="13"/>
+      <c r="I94" s="12"/>
     </row>
     <row r="95" spans="1:9" ht="15"/>
     <row r="96" spans="1:9" ht="15"/>
@@ -4042,6 +4035,7 @@
     <row r="99" ht="15"/>
     <row r="100" ht="15"/>
     <row r="101" ht="15"/>
+    <row r="102" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4052,17 +4046,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="1761f70d-44fd-470c-b684-9f606ffdaf59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bc6a1486-912e-4913-a829-15ae86dbf702">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000EE8C398961DF941AEC77EC2C80523D9" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1fc59492981de7ebc87db16151d63b13">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bc6a1486-912e-4913-a829-15ae86dbf702" xmlns:ns3="1761f70d-44fd-470c-b684-9f606ffdaf59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9959b8de82e23de46f65627169ae6472" ns2:_="" ns3:_="">
     <xsd:import namespace="bc6a1486-912e-4913-a829-15ae86dbf702"/>
@@ -4269,7 +4252,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -4278,14 +4261,25 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="1761f70d-44fd-470c-b684-9f606ffdaf59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bc6a1486-912e-4913-a829-15ae86dbf702">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A710723-3749-4100-8E4E-E30FEED8DF56}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A898D97-96D1-4B39-85DD-7745B6F800C6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A898D97-96D1-4B39-85DD-7745B6F800C6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71B6610F-9715-46B3-A0FF-F090E200262E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71B6610F-9715-46B3-A0FF-F090E200262E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A710723-3749-4100-8E4E-E30FEED8DF56}"/>
 </file>
</xml_diff>